<commit_message>
Record successful hosted Redot matrix
</commit_message>
<xml_diff>
--- a/docs/gamedev/source-of-truth.xlsx
+++ b/docs/gamedev/source-of-truth.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="R1788efd0c9ad43fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="Rdde41152fefb4877"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R22edcf9d780e49ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="Rd76cae528e444f33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Log" sheetId="5" r:id="R2381ab4663c544b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="6" r:id="Rfb296fc6c93b4162"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="R95ba507bd3964089"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Releases" sheetId="8" r:id="Rcf1c13d9dfb44726"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="9" r:id="R2941a68beedf43ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" r:id="Rabb8ae1d2d074e01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="2" r:id="R585879b2669d40e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R95664f3e5a6f4196"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Milestones" sheetId="4" r:id="R278b637f15be4c01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Build Log" sheetId="5" r:id="R3a8f1cd10c4a4ddd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="QA" sheetId="6" r:id="Reaa78e03b4fe4a68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks" sheetId="7" r:id="Raaf53374c37e451a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Releases" sheetId="8" r:id="Rdbbef4932b77432f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Marketing" sheetId="9" r:id="R1fca339a9f2341c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -157,8 +157,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="GameDev2" displayName="GameDev2" ref="A1:I18" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:I18"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="GameDev2" displayName="GameDev2" ref="A1:I19" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:I19"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date"/>
@@ -175,8 +175,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="GameDev3" displayName="GameDev3" ref="A1:Q33" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:Q33"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="GameDev3" displayName="GameDev3" ref="A1:Q34" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:Q34"/>
   <x:tableColumns count="17">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Title"/>
@@ -219,8 +219,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GameDev5" displayName="GameDev5" ref="A1:I13" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:I13"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="GameDev5" displayName="GameDev5" ref="A1:I14" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:I14"/>
   <x:tableColumns count="9">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date Time"/>
@@ -237,8 +237,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="GameDev6" displayName="GameDev6" ref="A1:K19" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:K19"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="GameDev6" displayName="GameDev6" ref="A1:K20" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:K20"/>
   <x:tableColumns count="11">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date Time"/>
@@ -276,8 +276,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="GameDev8" displayName="GameDev8" ref="A1:L3" headerRowCount="1" totalsRowCount="0">
-  <x:autoFilter ref="A1:L3"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="GameDev8" displayName="GameDev8" ref="A1:L4" headerRowCount="1" totalsRowCount="0">
+  <x:autoFilter ref="A1:L4"/>
   <x:tableColumns count="12">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Date Time"/>
@@ -649,20 +649,20 @@
         <x:v>Runtime tuple, API/interface hashes, native editor/release builds, integration suite, and export path are proven against the pinned Redot release</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="54" hidden="0" customHeight="1">
+    <x:row r="7" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A7" s="5" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">Status</x:t>
         </x:is>
       </x:c>
       <x:c r="B7" s="5" t="str">
-        <x:v>Latest v2.5 port is technically complete and validated locally on Redot 26.2; public name clearance and first hosted all-platform CI run remain external release gates</x:v>
+        <x:v>Latest v2.5 port is public and technically verified on Redot 26.2; the first hosted all-platform matrix passed with 19 successful jobs; tagged release remains gated by public-name clearance and explicit authorization</x:v>
       </x:c>
       <x:c r="C7" s="5" t="str">
         <x:v>2026-08-11</x:v>
       </x:c>
       <x:c r="D7" s="5" t="str">
-        <x:v>No external fork, tag, release, or publication has been created; explicit authorization is required immediately before that action</x:v>
+        <x:v>Public fork: https://github.com/dominicbytes/redotchestrator; hosted run: https://github.com/dominicbytes/redotchestrator/actions/runs/31560191202; no tag or GitHub release created</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
@@ -712,7 +712,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8bc7f9d7651b4407"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae4266d7bcf342ad"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1290,10 +1290,39 @@
         <x:v>DECISIONS.md#adr-0022-use-original-downstream-artwork</x:v>
       </x:c>
     </x:row>
+    <x:row r="19" ht="66" hidden="0" customHeight="1">
+      <x:c r="A19" s="3" t="str">
+        <x:v>DEC-043</x:v>
+      </x:c>
+      <x:c r="B19" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C19" s="3" t="str">
+        <x:v>Publication</x:v>
+      </x:c>
+      <x:c r="D19" s="3" t="str">
+        <x:v>Publish the verified port as the public dominicbytes/redotchestrator fork with redot-26.2 as its default branch, then require one green hosted matrix before release tagging.</x:v>
+      </x:c>
+      <x:c r="E19" s="3" t="str">
+        <x:v>The owner explicitly authorized repository publication; hosted platforms provide the missing cross-platform evidence.</x:v>
+      </x:c>
+      <x:c r="F19" s="3" t="str">
+        <x:v>Keep the work local or publish a source repository without hosted verification</x:v>
+      </x:c>
+      <x:c r="G19" s="3" t="str">
+        <x:v>Accepted</x:v>
+      </x:c>
+      <x:c r="H19" s="3" t="str">
+        <x:v>DominicBytes</x:v>
+      </x:c>
+      <x:c r="I19" s="3" t="str">
+        <x:v>https://github.com/dominicbytes/redotchestrator/actions/runs/31560191202</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R24f4ac1ef7c74ae1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81519c0abd9149cb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3114,10 +3143,63 @@
         <x:v>High</x:v>
       </x:c>
     </x:row>
+    <x:row r="34" ht="66" hidden="0" customHeight="1">
+      <x:c r="A34" s="3" t="str">
+        <x:v>SRC-032</x:v>
+      </x:c>
+      <x:c r="B34" s="3" t="str">
+        <x:v>First public redotchestrator hosted matrix</x:v>
+      </x:c>
+      <x:c r="C34" s="3" t="str">
+        <x:v>https://github.com/dominicbytes/redotchestrator/actions/runs/31560191202</x:v>
+      </x:c>
+      <x:c r="D34" s="3" t="str">
+        <x:v>CI run</x:v>
+      </x:c>
+      <x:c r="E34" s="3" t="str">
+        <x:v>GitHub Actions</x:v>
+      </x:c>
+      <x:c r="F34" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="G34" s="3" t="str">
+        <x:v>Redot 26.2</x:v>
+      </x:c>
+      <x:c r="H34" s="3" t="str">
+        <x:v>Linux, macOS, Windows, Android, Web, and iOS</x:v>
+      </x:c>
+      <x:c r="I34" s="3" t="str">
+        <x:v>Repository workflow evidence</x:v>
+      </x:c>
+      <x:c r="J34" s="3" t="str">
+        <x:v>Authoritative hosted platform and combined-artifact result</x:v>
+      </x:c>
+      <x:c r="K34" s="3" t="str">
+        <x:v>MS-032; MS-034</x:v>
+      </x:c>
+      <x:c r="L34" s="3" t="str">
+        <x:v>Commit 1ee46ff31a6a3e93ebb8c1d82897ee9c3d77c543 completed 19 jobs successfully; release job skipped correctly because no tag was pushed.</x:v>
+      </x:c>
+      <x:c r="M34" s="3" t="str">
+        <x:v>All descriptor targets and combined artifact jobs passed.</x:v>
+      </x:c>
+      <x:c r="N34" s="3" t="str">
+        <x:v>Downloaded plugin artifact 9127825011 and re-ran the strict package validator locally.</x:v>
+      </x:c>
+      <x:c r="O34" s="3" t="str">
+        <x:v>.out/hosted-artifacts/run-31560191202</x:v>
+      </x:c>
+      <x:c r="P34" s="3" t="str">
+        <x:v>Accept as hosted evidence</x:v>
+      </x:c>
+      <x:c r="Q34" s="3" t="str">
+        <x:v>High</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7133e2f2ceef4a81"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R77a6bc1e63a64174"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3454,7 +3536,7 @@
         <x:v>Feature-matrix fixtures; bounded editor/runtime runs; save/reopen comparisons; safe updater tests; platform export smoke tests; compatibility Gauntlet</x:v>
       </x:c>
       <x:c r="G10" s="5" t="str">
-        <x:v>In Progress</x:v>
+        <x:v>Completed</x:v>
       </x:c>
       <x:c r="H10" s="5" t="str">
         <x:v>Codex</x:v>
@@ -3466,7 +3548,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37134c9d99d44631"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1dd97c6ec244c73"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3897,10 +3979,39 @@
         <x:v>42/42 integration scenes; 1/1 native CTest; 4/4 package tests; clean workflow lint; both release runtime paths exited 0.</x:v>
       </x:c>
     </x:row>
+    <x:row r="14" ht="118.80000305175781" hidden="0" customHeight="1">
+      <x:c r="A14" s="3" t="str">
+        <x:v>BLD-020</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C14" s="3" t="str">
+        <x:v>Public fork and first hosted matrix</x:v>
+      </x:c>
+      <x:c r="D14" s="3" t="str">
+        <x:v>Created the public downstream fork, pushed redot-26.2, made it the default branch, completed the full hosted matrix, and downloaded/validated the combined plugin artifact.</x:v>
+      </x:c>
+      <x:c r="E14" s="3" t="str">
+        <x:v>https://github.com/dominicbytes/redotchestrator; .out/hosted-artifacts/run-31560191202</x:v>
+      </x:c>
+      <x:c r="F14" s="3" t="str">
+        <x:v>1ee46ff31a6a3e93ebb8c1d82897ee9c3d77c543</x:v>
+      </x:c>
+      <x:c r="G14" s="3" t="str">
+        <x:v>GitHub fork-parent/default-branch/ref checks; 19-job matrix; artifact digest; strict package validation</x:v>
+      </x:c>
+      <x:c r="H14" s="3" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="I14" s="3" t="str">
+        <x:v>Run 31560191202; plugin artifact 9127825011 digest sha256:9b3b82d45a6333caa2914f8141d1d76978903dbb355d91cafe8d8c239b4144a6; generated package SHA-256 768d6805f0ffa1edac64cfe1403d99f506ac65e2110be284c0114fc85ae9dec2.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R84350c01a0114db6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R299cb6fa62a34228"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4631,10 +4742,45 @@
         <x:v>Codex</x:v>
       </x:c>
     </x:row>
+    <x:row r="20" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A20" s="3" t="str">
+        <x:v>QA-026</x:v>
+      </x:c>
+      <x:c r="B20" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C20" s="3" t="str">
+        <x:v>MS-032; MS-034 hosted closure</x:v>
+      </x:c>
+      <x:c r="D20" s="3" t="str">
+        <x:v>Run every advertised platform build, combine artifacts, download the universal plugin artifact, and execute the strict release packager</x:v>
+      </x:c>
+      <x:c r="E20" s="3" t="str">
+        <x:v>GitHub-hosted Linux, macOS, Windows, Android, Web, and iOS runners; commit 1ee46ff3</x:v>
+      </x:c>
+      <x:c r="F20" s="3" t="str">
+        <x:v>All platform and assembly jobs pass; the downloaded artifact contains every descriptor library and packages deterministically</x:v>
+      </x:c>
+      <x:c r="G20" s="3" t="str">
+        <x:v>PASS: 19 jobs succeeded; plugin/demo artifacts uploaded; downloaded plugin packaged at 53,367,796 bytes with SHA-256 768d6805f0ffa1edac64cfe1403d99f506ac65e2110be284c0114fc85ae9dec2</x:v>
+      </x:c>
+      <x:c r="H20" s="3" t="str">
+        <x:v>https://github.com/dominicbytes/redotchestrator/actions/runs/31560191202; UPSTREAM_LOCK.md</x:v>
+      </x:c>
+      <x:c r="I20" s="3" t="str">
+        <x:v>Critical</x:v>
+      </x:c>
+      <x:c r="J20" s="3" t="str">
+        <x:v>Passed</x:v>
+      </x:c>
+      <x:c r="K20" s="3" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf435de62f714a62"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R112602785bcc4955"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4840,13 +4986,13 @@
         <x:v>May block a public or reproducible Redot release.</x:v>
       </x:c>
       <x:c r="F5" s="5" t="str">
-        <x:v>Create the public fork only after the user gives explicit publication authorization.</x:v>
+        <x:v>The owner authorized publication and the public fork now exists with redot-26.2 as its default branch.</x:v>
       </x:c>
       <x:c r="G5" s="5" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H5" s="5" t="str">
-        <x:v>Open</x:v>
+        <x:v>Closed</x:v>
       </x:c>
       <x:c r="I5" s="5" t="str">
         <x:v>Before port baseline</x:v>
@@ -5032,13 +5178,13 @@
         <x:v>High: upstream CI primarily runs integration tests on Linux x86_64 while other platforms are build-only.</x:v>
       </x:c>
       <x:c r="F11" s="5" t="str">
-        <x:v>The complete matrix is fail-closed, but the first hosted Linux/macOS/Windows/Android/Web/iOS execution is still required.</x:v>
+        <x:v>The first complete hosted matrix passed all platform builds and combined artifact assembly; platform-specific runtime depth remains governed by each available runner.</x:v>
       </x:c>
       <x:c r="G11" s="5" t="str">
         <x:v>Codex</x:v>
       </x:c>
       <x:c r="H11" s="5" t="str">
-        <x:v>Open</x:v>
+        <x:v>Mitigated</x:v>
       </x:c>
       <x:c r="I11" s="5" t="str">
         <x:v>Before release candidate</x:v>
@@ -5242,7 +5388,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad22bd8713554be8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc7896c7142ca4b61"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5418,19 +5564,57 @@
         <x:v>42/42 integration; CTest 1/1; package 4/4; actionlint; release/export exit 0</x:v>
       </x:c>
       <x:c r="J3" s="3" t="str">
-        <x:v>Local Windows candidate; GitHub-hosted universal artifact pending</x:v>
+        <x:v>Historical local candidate; superseded by hosted candidate REL-002</x:v>
       </x:c>
       <x:c r="K3" s="3" t="str">
         <x:v>Validated Locally</x:v>
       </x:c>
       <x:c r="L3" s="3" t="str">
-        <x:v>No publication performed. Redot name clearance and the first hosted all-platform matrix remain external release gates.</x:v>
+        <x:v>Pre-publication Windows evidence retained for provenance; see REL-002 for the public fork and hosted matrix.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="105.5999984741211" hidden="0" customHeight="1">
+      <x:c r="A4" s="3" t="str">
+        <x:v>REL-002</x:v>
+      </x:c>
+      <x:c r="B4" s="3" t="str">
+        <x:v>2026-08-11</x:v>
+      </x:c>
+      <x:c r="C4" s="3" t="str">
+        <x:v>v2.5.stable pre-tag candidate</x:v>
+      </x:c>
+      <x:c r="D4" s="3" t="str">
+        <x:v>1ee46ff31a6a3e93ebb8c1d82897ee9c3d77c543</x:v>
+      </x:c>
+      <x:c r="E4" s="3" t="str">
+        <x:v>Linux, macOS, Windows, Android, Web, and iOS</x:v>
+      </x:c>
+      <x:c r="F4" s="3" t="str">
+        <x:v>redotchestrator CI run 31560191202</x:v>
+      </x:c>
+      <x:c r="G4" s="3" t="str">
+        <x:v>GitHub artifacts 9127825011 redotchestrator-plugin; 9127825442 redotchestrator-demo; locally generated validated package</x:v>
+      </x:c>
+      <x:c r="H4" s="3" t="str">
+        <x:v>plugin artifact sha256:9b3b82d45a6333caa2914f8141d1d76978903dbb355d91cafe8d8c239b4144a6; package sha256:768d6805f0ffa1edac64cfe1403d99f506ac65e2110be284c0114fc85ae9dec2</x:v>
+      </x:c>
+      <x:c r="I4" s="3" t="str">
+        <x:v>19 hosted jobs succeeded; strict package validation passed after download</x:v>
+      </x:c>
+      <x:c r="J4" s="3" t="str">
+        <x:v>https://github.com/dominicbytes/redotchestrator/actions/runs/31560191202</x:v>
+      </x:c>
+      <x:c r="K4" s="3" t="str">
+        <x:v>Hosted Matrix Passed</x:v>
+      </x:c>
+      <x:c r="L4" s="3" t="str">
+        <x:v>No release tag published; Redot name clearance and explicit release authorization remain required.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4768b025fbac429c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re1858c9c2a9941d1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5646,7 +5830,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd363b8c471cd48d2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a3595b3adc34e10"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>